<commit_message>
Refresh demo outputs from the PR's LibreOffice-backed CI run
Downloaded from the regenerated-artifacts upload of CI run 35886975862 on 2887803. The demo reports carry the same 13 findings; they now show the LIVE_ERROR formula and the reworded FORMULA_DRIFT fix, and the regenerated demo workbook has a new hash. The seeded-defect matrix is unchanged.
</commit_message>
<xml_diff>
--- a/examples/demo_annotated.xlsx
+++ b/examples/demo_annotated.xlsx
@@ -142,16 +142,22 @@
   <commentList>
     <comment ref="B6" authorId="0" shapeId="0">
       <text>
-        <t>High TOTAL_MISMATCH
+        <t>High FORMULA_DRIFT
+Formula breaks neighboring pattern
+Fix: If this cell is the same kind of line as its neighbors, restore their pattern. A total, net or summary line differs by design: compare it with the other totals instead.
+High TOTAL_MISMATCH
 Total double-counts a cell inside its own range
 Fix: Remove the duplicated term or shrink the range so each component is counted once.</t>
       </text>
     </comment>
     <comment ref="E6" authorId="0" shapeId="0">
       <text>
-        <t>High FORMULA_DRIFT
+        <t>Critical CROSS_FOOT_FAILURE
+Row totals and column totals disagree
+Fix: Reconcile the totals row and totals column; one of the contributing aggregates is likely wrong.
+High FORMULA_DRIFT
 Formula breaks neighboring pattern
-Fix: Compare this formula to adjacent formulas and restore the intended relative references.</t>
+Fix: If this cell is the same kind of line as its neighbors, restore their pattern. A total, net or summary line differs by design: compare it with the other totals instead.</t>
       </text>
     </comment>
     <comment ref="E9" authorId="0" shapeId="0">
@@ -163,9 +169,12 @@
     </comment>
     <comment ref="B10" authorId="0" shapeId="0">
       <text>
-        <t>High FORMULA_DRIFT
+        <t>Critical RANGE_EXCLUSION
+Aggregation range appears to exclude adjacent data row
+Fix: Confirm whether Budget!B9 belongs in the aggregate, then extend the range if appropriate.
+High FORMULA_DRIFT
 Formula breaks neighboring pattern
-Fix: Compare this formula to adjacent formulas and restore the intended relative references.</t>
+Fix: If this cell is the same kind of line as its neighbors, restore their pattern. A total, net or summary line differs by design: compare it with the other totals instead.</t>
       </text>
     </comment>
     <comment ref="B13" authorId="0" shapeId="0">
@@ -177,7 +186,10 @@
     </comment>
     <comment ref="B14" authorId="0" shapeId="0">
       <text>
-        <t>High BROKEN_REFERENCE
+        <t>Critical LIVE_ERROR
+Cell contains live spreadsheet error
+Fix: Trace the formula precedent chain and resolve the underlying spreadsheet error.
+High BROKEN_REFERENCE
 Formula contains deleted reference
 Fix: Restore the deleted reference or rebuild the formula from intended source cells.</t>
       </text>

</xml_diff>

<commit_message>
Refresh the demo outputs and seeded matrix from a LibreOffice-backed run
Regenerated by CI with recalculation available. The demo report, HTML and findings JSON show 0.4.0 output: the audit status line, content fingerprints with the pinned line to accept each finding, members, and coverage.complete. The seeded matrix carries the new IFERROR_MASK case note; every seeded defect is detected, with no unexpected findings.
</commit_message>
<xml_diff>
--- a/examples/demo_annotated.xlsx
+++ b/examples/demo_annotated.xlsx
@@ -198,21 +198,24 @@
       <text>
         <t>Medium DUPLICATE_KEY
 Duplicate key in lookup range
-Fix: Make the keys unique or confirm the lookup is meant to return the first match.</t>
+Fix: Make the keys unique or confirm the lookup is meant to return the first match.
+The same issue is in 1 other cell(s); fixing it here usually fixes them.</t>
       </text>
     </comment>
     <comment ref="A18" authorId="0" shapeId="0">
       <text>
-        <t>Medium WHITESPACE_KEY
+        <t>Medium DUPLICATE_KEY
+Same issue as Budget!A17, Budget!A18; see the comment there.
+Medium WHITESPACE_KEY
 Text has leading or trailing whitespace
-Fix: Trim the value if it is used as a lookup key or label.</t>
+Fix: Trim the values if they are used as lookup keys or labels.</t>
       </text>
     </comment>
     <comment ref="B20" authorId="0" shapeId="0">
       <text>
         <t>High NUMBERS_STORED_AS_TEXT
 Numeric-looking value stored as text
-Fix: Convert the value to a number or confirm it is intentionally text.</t>
+Fix: Convert the values to numbers or confirm they are intentionally text.</t>
       </text>
     </comment>
   </commentList>

</xml_diff>